<commit_message>
Minor fixes, additional selectors and logic added, error handling part 1
</commit_message>
<xml_diff>
--- a/samples/sample_procurement.xlsx
+++ b/samples/sample_procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual Studios Repos\Chaman\RPA_BOT\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22BD4F8D-80D3-4DF2-AD73-0FFD0340382F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46B36E79-5986-4A9D-B5EB-81037B1A5230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Finance Year</t>
   </si>
@@ -52,31 +52,40 @@
     <t>Domestically</t>
   </si>
   <si>
-    <t>Sample Tyre Supplier Pvt Ltd</t>
-  </si>
-  <si>
     <t>Scrap tyre/used tyre/cut tyre</t>
   </si>
   <si>
-    <t>PROC-001</t>
-  </si>
-  <si>
-    <t>27ABCDE1234F1Z5</t>
-  </si>
-  <si>
-    <t>01/04/2026</t>
-  </si>
-  <si>
-    <t>PROC-001.pdf</t>
-  </si>
-  <si>
     <t>2026-2027</t>
+  </si>
+  <si>
+    <t>Contact Details</t>
+  </si>
+  <si>
+    <t>Address of waste tyre supplier</t>
+  </si>
+  <si>
+    <t>98181 45119</t>
+  </si>
+  <si>
+    <t>JAI AMBEY TRADERS</t>
+  </si>
+  <si>
+    <t>CW - 575, Sanjay Gandhi Transport Nagar, Delhi - 110042</t>
+  </si>
+  <si>
+    <t>07CELPK9227A1ZJ</t>
+  </si>
+  <si>
+    <t>shree sai 045.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -104,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -112,13 +121,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,20 +447,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="32" customWidth="1"/>
-    <col min="5" max="5" width="31" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="25" customWidth="1"/>
-    <col min="8" max="9" width="19" customWidth="1"/>
+    <col min="3" max="5" width="31" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="31" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="15.44140625" customWidth="1"/>
+    <col min="11" max="11" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -445,51 +472,63 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2">
-        <v>12.5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
+      <c r="G2" s="2">
+        <v>3.82</v>
+      </c>
+      <c r="H2" s="2">
+        <v>45</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3">
+        <v>46182</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>